<commit_message>
Complete Chapter 4 Stand
</commit_message>
<xml_diff>
--- a/Results/Jump/DetectedAction/FindPrincipalComponents_PipelinePCA_Jump/PCA_Dimension_Search_PipelinePCA.xlsx
+++ b/Results/Jump/DetectedAction/FindPrincipalComponents_PipelinePCA_Jump/PCA_Dimension_Search_PipelinePCA.xlsx
@@ -1090,40 +1090,40 @@
         <v>40</v>
       </c>
       <c r="B12" t="n">
-        <v>88.00000000000001</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="C12" t="n">
-        <v>89.69841269841272</v>
+        <v>91.03174603174604</v>
       </c>
       <c r="D12" t="n">
-        <v>87.99999999999999</v>
+        <v>89.33333333333331</v>
       </c>
       <c r="E12" t="n">
-        <v>94</v>
+        <v>94.66666666666667</v>
       </c>
       <c r="F12" t="n">
-        <v>88.09427609427608</v>
+        <v>89.42760942760944</v>
       </c>
       <c r="G12" t="n">
-        <v>87.99999999999999</v>
+        <v>89.33333333333331</v>
       </c>
       <c r="H12" t="n">
-        <v>7.774602526460403</v>
+        <v>8.000000000000004</v>
       </c>
       <c r="I12" t="n">
-        <v>6.678070367607634</v>
+        <v>6.825396825396833</v>
       </c>
       <c r="J12" t="n">
-        <v>7.774602526460393</v>
+        <v>7.999999999999995</v>
       </c>
       <c r="K12" t="n">
-        <v>3.8873012632302</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>7.470487456551007</v>
+        <v>7.676767676767682</v>
       </c>
       <c r="M12" t="n">
-        <v>7.774602526460393</v>
+        <v>7.999999999999995</v>
       </c>
     </row>
     <row r="13">
@@ -1254,40 +1254,40 @@
         <v>36</v>
       </c>
       <c r="B16" t="n">
-        <v>88.00000000000001</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="C16" t="n">
-        <v>89.69841269841272</v>
+        <v>91.03174603174604</v>
       </c>
       <c r="D16" t="n">
-        <v>87.99999999999999</v>
+        <v>89.33333333333331</v>
       </c>
       <c r="E16" t="n">
-        <v>94</v>
+        <v>94.66666666666667</v>
       </c>
       <c r="F16" t="n">
-        <v>88.09427609427608</v>
+        <v>89.42760942760944</v>
       </c>
       <c r="G16" t="n">
-        <v>87.99999999999999</v>
+        <v>89.33333333333331</v>
       </c>
       <c r="H16" t="n">
-        <v>7.774602526460403</v>
+        <v>8.000000000000004</v>
       </c>
       <c r="I16" t="n">
-        <v>6.678070367607634</v>
+        <v>6.825396825396833</v>
       </c>
       <c r="J16" t="n">
-        <v>7.774602526460393</v>
+        <v>7.999999999999995</v>
       </c>
       <c r="K16" t="n">
-        <v>3.8873012632302</v>
+        <v>4</v>
       </c>
       <c r="L16" t="n">
-        <v>7.470487456551007</v>
+        <v>7.676767676767682</v>
       </c>
       <c r="M16" t="n">
-        <v>7.774602526460393</v>
+        <v>7.999999999999995</v>
       </c>
     </row>
     <row r="17">
@@ -1459,40 +1459,40 @@
         <v>31</v>
       </c>
       <c r="B21" t="n">
-        <v>89.33333333333333</v>
+        <v>90.66666666666669</v>
       </c>
       <c r="C21" t="n">
-        <v>91.03174603174604</v>
+        <v>91.66666666666667</v>
       </c>
       <c r="D21" t="n">
-        <v>89.33333333333331</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="E21" t="n">
-        <v>94.66666666666667</v>
+        <v>95.33333333333334</v>
       </c>
       <c r="F21" t="n">
-        <v>89.42760942760944</v>
+        <v>90.57239057239057</v>
       </c>
       <c r="G21" t="n">
-        <v>89.33333333333331</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="H21" t="n">
-        <v>8.000000000000004</v>
+        <v>5.333333333333333</v>
       </c>
       <c r="I21" t="n">
-        <v>6.825396825396833</v>
+        <v>5.555555555555562</v>
       </c>
       <c r="J21" t="n">
-        <v>7.999999999999995</v>
+        <v>5.333333333333332</v>
       </c>
       <c r="K21" t="n">
-        <v>4</v>
+        <v>2.666666666666666</v>
       </c>
       <c r="L21" t="n">
-        <v>7.676767676767682</v>
+        <v>5.387205387205385</v>
       </c>
       <c r="M21" t="n">
-        <v>7.999999999999995</v>
+        <v>5.333333333333332</v>
       </c>
     </row>
     <row r="22">
@@ -1544,37 +1544,37 @@
         <v>89.33333333333333</v>
       </c>
       <c r="C23" t="n">
-        <v>91.03174603174604</v>
+        <v>90.33333333333336</v>
       </c>
       <c r="D23" t="n">
-        <v>89.33333333333331</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="E23" t="n">
         <v>94.66666666666667</v>
       </c>
       <c r="F23" t="n">
-        <v>89.42760942760944</v>
+        <v>89.23905723905723</v>
       </c>
       <c r="G23" t="n">
-        <v>89.33333333333331</v>
+        <v>89.33333333333333</v>
       </c>
       <c r="H23" t="n">
-        <v>8.000000000000004</v>
+        <v>5.333333333333331</v>
       </c>
       <c r="I23" t="n">
-        <v>6.825396825396833</v>
+        <v>5.528824579833219</v>
       </c>
       <c r="J23" t="n">
-        <v>7.999999999999995</v>
+        <v>5.333333333333331</v>
       </c>
       <c r="K23" t="n">
-        <v>4</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="L23" t="n">
-        <v>7.676767676767682</v>
+        <v>5.38053459042612</v>
       </c>
       <c r="M23" t="n">
-        <v>7.999999999999995</v>
+        <v>5.333333333333331</v>
       </c>
     </row>
     <row r="24">
@@ -1746,40 +1746,40 @@
         <v>24</v>
       </c>
       <c r="B28" t="n">
-        <v>92.00000000000001</v>
+        <v>90.66666666666669</v>
       </c>
       <c r="C28" t="n">
-        <v>92.77777777777779</v>
+        <v>91.66666666666667</v>
       </c>
       <c r="D28" t="n">
-        <v>92</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="E28" t="n">
-        <v>96</v>
+        <v>95.33333333333334</v>
       </c>
       <c r="F28" t="n">
-        <v>91.91919191919192</v>
+        <v>90.57239057239057</v>
       </c>
       <c r="G28" t="n">
-        <v>92</v>
+        <v>90.66666666666666</v>
       </c>
       <c r="H28" t="n">
-        <v>6.531972647421807</v>
+        <v>5.333333333333333</v>
       </c>
       <c r="I28" t="n">
-        <v>6.478835438717005</v>
+        <v>5.555555555555562</v>
       </c>
       <c r="J28" t="n">
-        <v>6.53197264742181</v>
+        <v>5.333333333333332</v>
       </c>
       <c r="K28" t="n">
-        <v>3.265986323710904</v>
+        <v>2.666666666666666</v>
       </c>
       <c r="L28" t="n">
-        <v>6.597952169112936</v>
+        <v>5.387205387205385</v>
       </c>
       <c r="M28" t="n">
-        <v>6.53197264742181</v>
+        <v>5.333333333333332</v>
       </c>
     </row>
     <row r="29">
@@ -2197,40 +2197,40 @@
         <v>13</v>
       </c>
       <c r="B39" t="n">
-        <v>90.66666666666669</v>
+        <v>92.00000000000001</v>
       </c>
       <c r="C39" t="n">
-        <v>91.66666666666667</v>
+        <v>92.77777777777779</v>
       </c>
       <c r="D39" t="n">
-        <v>90.66666666666666</v>
+        <v>92</v>
       </c>
       <c r="E39" t="n">
-        <v>95.33333333333334</v>
+        <v>96</v>
       </c>
       <c r="F39" t="n">
-        <v>90.57239057239057</v>
+        <v>91.91919191919192</v>
       </c>
       <c r="G39" t="n">
-        <v>90.66666666666666</v>
+        <v>92</v>
       </c>
       <c r="H39" t="n">
-        <v>5.333333333333333</v>
+        <v>6.531972647421806</v>
       </c>
       <c r="I39" t="n">
-        <v>5.555555555555562</v>
+        <v>6.478835438717005</v>
       </c>
       <c r="J39" t="n">
-        <v>5.333333333333332</v>
+        <v>6.53197264742181</v>
       </c>
       <c r="K39" t="n">
-        <v>2.666666666666666</v>
+        <v>3.265986323710903</v>
       </c>
       <c r="L39" t="n">
-        <v>5.387205387205385</v>
+        <v>6.597952169112936</v>
       </c>
       <c r="M39" t="n">
-        <v>5.333333333333332</v>
+        <v>6.53197264742181</v>
       </c>
     </row>
     <row r="40">
@@ -4193,22 +4193,22 @@
         <v>5</v>
       </c>
       <c r="C56" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="D56" t="n">
-        <v>87.77777777777777</v>
+        <v>94.44444444444446</v>
       </c>
       <c r="E56" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="F56" t="n">
-        <v>93.33333333333333</v>
+        <v>96.66666666666667</v>
       </c>
       <c r="G56" t="n">
-        <v>86.5993265993266</v>
+        <v>93.26599326599326</v>
       </c>
       <c r="H56" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="57">
@@ -4713,22 +4713,22 @@
         <v>5</v>
       </c>
       <c r="C76" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="D76" t="n">
-        <v>87.77777777777777</v>
+        <v>94.44444444444446</v>
       </c>
       <c r="E76" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="F76" t="n">
-        <v>93.33333333333333</v>
+        <v>96.66666666666667</v>
       </c>
       <c r="G76" t="n">
-        <v>86.5993265993266</v>
+        <v>93.26599326599326</v>
       </c>
       <c r="H76" t="n">
-        <v>86.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="77">
@@ -5285,22 +5285,22 @@
         <v>2</v>
       </c>
       <c r="C98" t="n">
-        <v>73.33333333333333</v>
+        <v>80</v>
       </c>
       <c r="D98" t="n">
-        <v>77.38095238095238</v>
+        <v>80.55555555555554</v>
       </c>
       <c r="E98" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F98" t="n">
-        <v>86.66666666666667</v>
+        <v>90</v>
       </c>
       <c r="G98" t="n">
-        <v>74.07407407407406</v>
+        <v>79.79797979797981</v>
       </c>
       <c r="H98" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
     </row>
     <row r="99">
@@ -5545,22 +5545,22 @@
         <v>2</v>
       </c>
       <c r="C108" t="n">
-        <v>73.33333333333333</v>
+        <v>80</v>
       </c>
       <c r="D108" t="n">
-        <v>77.38095238095238</v>
+        <v>80.55555555555554</v>
       </c>
       <c r="E108" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
       <c r="F108" t="n">
-        <v>86.66666666666667</v>
+        <v>90</v>
       </c>
       <c r="G108" t="n">
-        <v>74.07407407407406</v>
+        <v>79.79797979797981</v>
       </c>
       <c r="H108" t="n">
-        <v>73.33333333333334</v>
+        <v>80</v>
       </c>
     </row>
     <row r="109">
@@ -5623,22 +5623,22 @@
         <v>5</v>
       </c>
       <c r="C111" t="n">
-        <v>93.33333333333333</v>
+        <v>86.66666666666667</v>
       </c>
       <c r="D111" t="n">
-        <v>94.44444444444446</v>
+        <v>87.77777777777777</v>
       </c>
       <c r="E111" t="n">
-        <v>93.33333333333333</v>
+        <v>86.66666666666667</v>
       </c>
       <c r="F111" t="n">
-        <v>96.66666666666667</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="G111" t="n">
-        <v>93.26599326599326</v>
+        <v>86.5993265993266</v>
       </c>
       <c r="H111" t="n">
-        <v>93.33333333333333</v>
+        <v>86.66666666666667</v>
       </c>
     </row>
     <row r="112">
@@ -6247,22 +6247,22 @@
         <v>4</v>
       </c>
       <c r="C135" t="n">
-        <v>100</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="D135" t="n">
-        <v>100</v>
+        <v>94.44444444444446</v>
       </c>
       <c r="E135" t="n">
-        <v>100</v>
+        <v>93.33333333333333</v>
       </c>
       <c r="F135" t="n">
-        <v>100</v>
+        <v>96.66666666666667</v>
       </c>
       <c r="G135" t="n">
-        <v>100</v>
+        <v>93.26599326599326</v>
       </c>
       <c r="H135" t="n">
-        <v>100</v>
+        <v>93.33333333333333</v>
       </c>
     </row>
     <row r="136">
@@ -7651,22 +7651,22 @@
         <v>3</v>
       </c>
       <c r="C189" t="n">
-        <v>93.33333333333333</v>
+        <v>100</v>
       </c>
       <c r="D189" t="n">
-        <v>94.44444444444446</v>
+        <v>100</v>
       </c>
       <c r="E189" t="n">
-        <v>93.33333333333333</v>
+        <v>100</v>
       </c>
       <c r="F189" t="n">
-        <v>96.66666666666667</v>
+        <v>100</v>
       </c>
       <c r="G189" t="n">
-        <v>93.26599326599326</v>
+        <v>100</v>
       </c>
       <c r="H189" t="n">
-        <v>93.33333333333333</v>
+        <v>100</v>
       </c>
     </row>
     <row r="190">

</xml_diff>